<commit_message>
Tiered-claims master: add the neutrino Koide prediction (Q_ν≈0.77, toy-map extrapolation — flagged NOT ED-derived) to Core Predictions + Ledger; add the Koide re-description as an Inherited/Consilience ledger row; Tier Counts Prediction 24→25
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ED_TheoryList_TieredClaims.xlsx
+++ b/ED_TheoryList_TieredClaims.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Ratio" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ledger w Claims'!$A$1:$J$402</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ledger w Claims'!$A$1:$J$407</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tier Key'!$A$1:$E$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1535,7 +1535,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="14" customWidth="1" style="39" min="1" max="1"/>
@@ -2026,6 +2026,33 @@
       <c r="E18" s="40" t="inlineStr">
         <is>
           <t>resistivity saturation and the viscosity floor onset at different substrate occupancies (no correlation); or a second inter-locus transport channel exists beyond the P05/Adjacency band (F-BAND). Exact ratio needs Pi_p,Pi_q (open); MIR value inherited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="40" t="inlineStr">
+        <is>
+          <t>substrate-evaluation</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t>Koide</t>
+        </is>
+      </c>
+      <c r="C19" s="40" t="inlineStr">
+        <is>
+          <t>Neutrino Koide Q_nu = (m1+m2+m3)/(sqrt m1+sqrt m2+sqrt m3)^2 ~ 0.77 (TOY-MAP extrapolation over charge and isospin x hypercharge; wobble w~1.63). NOT ED-derived.</t>
+        </is>
+      </c>
+      <c r="D19" s="40" t="inlineStr">
+        <is>
+          <t>Prediction</t>
+        </is>
+      </c>
+      <c r="E19" s="40" t="inlineStr">
+        <is>
+          <t>Measured absolute neutrino masses whose Koide combination departs from ~0.77 refute the toy map. Untestable until absolute nu masses known. TOY-MODEL corner, not a derived ED prediction.</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J405"/>
+  <dimension ref="A1:J407"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18.71" customWidth="1" style="39" min="1" max="1"/>
@@ -18083,8 +18110,94 @@
         </is>
       </c>
     </row>
-    <row r="406" ht="15.75" customHeight="1" s="39"/>
-    <row r="407" ht="15.75" customHeight="1" s="39"/>
+    <row r="406" ht="15.75" customHeight="1" s="39">
+      <c r="A406" s="41" t="inlineStr">
+        <is>
+          <t>substrate-evaluation</t>
+        </is>
+      </c>
+      <c r="B406" s="41" t="inlineStr">
+        <is>
+          <t>Koide</t>
+        </is>
+      </c>
+      <c r="C406" s="41" t="inlineStr">
+        <is>
+          <t>Neutrino Koide Q_nu ~ 0.77 (TOY-MAP extrapolation; wobble w~1.63; both the charge and isospin x hypercharge maps agree). NOT ED-derived.</t>
+        </is>
+      </c>
+      <c r="D406" s="41" t="inlineStr">
+        <is>
+          <t>Prediction</t>
+        </is>
+      </c>
+      <c r="E406" s="41" t="inlineStr">
+        <is>
+          <t>measured absolute nu masses with Koide combination != ~0.77 refute; untestable until absolute nu masses known</t>
+        </is>
+      </c>
+      <c r="F406" s="41" t="inlineStr">
+        <is>
+          <t>toy-map extrapolation; not derived (masses inherited)</t>
+        </is>
+      </c>
+      <c r="G406" s="41" t="inlineStr">
+        <is>
+          <t>absolute nu masses unknown; untestable now</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>toy-model / re-description tier (Paper_Koide_GenerationCoherenceMap)</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr"/>
+      <c r="J406" t="inlineStr"/>
+    </row>
+    <row r="407" ht="15.75" customHeight="1" s="39">
+      <c r="A407" s="41" t="inlineStr">
+        <is>
+          <t>substrate-evaluation</t>
+        </is>
+      </c>
+      <c r="B407" s="41" t="inlineStr">
+        <is>
+          <t>Koide</t>
+        </is>
+      </c>
+      <c r="C407" s="41" t="inlineStr">
+        <is>
+          <t>Koide 2/3 re-described in ED amplitude/coherence language (mass = bandwidth b, sqrt m = amplitude): Q reads as a coherence ratio among 3 generation-amplitudes; Q = 1/3 + w^2/6; Brannen Z3 / sqrt2 form; leptons w=sqrt2, delta~2/9. RE-DESCRIPTION + consilience (masses organize like amplitudes), NOT a derivation.</t>
+        </is>
+      </c>
+      <c r="D407" s="41" t="inlineStr">
+        <is>
+          <t>Inherited / Consilience</t>
+        </is>
+      </c>
+      <c r="E407" s="41" t="inlineStr">
+        <is>
+          <t>n/a (re-description; no ED derivation to falsify)</t>
+        </is>
+      </c>
+      <c r="F407" s="41" t="inlineStr">
+        <is>
+          <t>none - re-description; mass sector inherited/open</t>
+        </is>
+      </c>
+      <c r="G407" s="41" t="inlineStr">
+        <is>
+          <t>generation count, masses, 2/3, w=sqrt2, delta~2/9 all inherited/open</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>referee-vetted; obeys B4 retrofit discipline; Paper_Koide_GenerationCoherenceMap</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr"/>
+      <c r="J407" t="inlineStr"/>
+    </row>
     <row r="408" ht="15.75" customHeight="1" s="39"/>
     <row r="409" ht="15.75" customHeight="1" s="39"/>
     <row r="410" ht="15.75" customHeight="1" s="39"/>
@@ -18679,7 +18792,7 @@
     <row r="999" ht="15.75" customHeight="1" s="39"/>
     <row r="1000" ht="15.75" customHeight="1" s="39"/>
   </sheetData>
-  <autoFilter ref="$A$1:$J$402">
+  <autoFilter ref="A1:J407">
     <sortState ref="A1:J402">
       <sortCondition ref="D1:D402"/>
       <sortCondition ref="J1:J402"/>
@@ -24607,12 +24720,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:B8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="43.43" customWidth="1" style="39" min="1" max="1"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="A2" s="33" t="inlineStr">
         <is>
@@ -24640,7 +24754,7 @@
         </is>
       </c>
       <c r="B4" s="33" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Koide: retire from EDG — move paper to the private event-density repo
The toy neutrino-corner prediction (Q_nu ~ 0.77) is disfavored by the
measured oscillation splittings (Q_nu <= 0.59 NO / 0.50 IO for any lightest
mass), so the paper is pulled from public EDG to the working repo. Drop the
PAPERS_INDEX pointer and remove the two Koide rows (disfavored neutrino
prediction + the ED re-description) from the public tiered-claims master;
live Prediction count 25 -> 24. The rigid charged-lepton 2/3 is untouched.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ED_TheoryList_TieredClaims.xlsx
+++ b/ED_TheoryList_TieredClaims.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Core Theory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Core Predictions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Ledger w Claims" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Core Claims" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Tier Key" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Tier Counts" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Postulate Flags" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Ratio" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Theory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Predictions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger w Claims" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Claims" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier Key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier Counts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Postulate Flags" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratio" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ledger w Claims'!$A$1:$J$407</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ledger w Claims'!$A$1:$J$405</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tier Key'!$A$1:$E$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1535,7 +1535,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="14" customWidth="1" style="39" min="1" max="1"/>
@@ -2026,33 +2026,6 @@
       <c r="E18" s="40" t="inlineStr">
         <is>
           <t>resistivity saturation and the viscosity floor onset at different substrate occupancies (no correlation); or a second inter-locus transport channel exists beyond the P05/Adjacency band (F-BAND). Exact ratio needs Pi_p,Pi_q (open); MIR value inherited.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="40" t="inlineStr">
-        <is>
-          <t>substrate-evaluation</t>
-        </is>
-      </c>
-      <c r="B19" s="40" t="inlineStr">
-        <is>
-          <t>Koide</t>
-        </is>
-      </c>
-      <c r="C19" s="40" t="inlineStr">
-        <is>
-          <t>Neutrino Koide Q_nu = (m1+m2+m3)/(sqrt m1+sqrt m2+sqrt m3)^2 ~ 0.77 (TOY-MAP extrapolation over charge and isospin x hypercharge; wobble w~1.63). NOT ED-derived.</t>
-        </is>
-      </c>
-      <c r="D19" s="40" t="inlineStr">
-        <is>
-          <t>Prediction</t>
-        </is>
-      </c>
-      <c r="E19" s="40" t="inlineStr">
-        <is>
-          <t>Measured absolute neutrino masses whose Koide combination departs from ~0.77 refute the toy map. Untestable until absolute nu masses known. TOY-MODEL corner, not a derived ED prediction.</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J407"/>
+  <dimension ref="A1:J405"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18.71" customWidth="1" style="39" min="1" max="1"/>
@@ -18110,94 +18083,8 @@
         </is>
       </c>
     </row>
-    <row r="406" ht="15.75" customHeight="1" s="39">
-      <c r="A406" s="41" t="inlineStr">
-        <is>
-          <t>substrate-evaluation</t>
-        </is>
-      </c>
-      <c r="B406" s="41" t="inlineStr">
-        <is>
-          <t>Koide</t>
-        </is>
-      </c>
-      <c r="C406" s="41" t="inlineStr">
-        <is>
-          <t>Neutrino Koide Q_nu ~ 0.77 (TOY-MAP extrapolation; wobble w~1.63; both the charge and isospin x hypercharge maps agree). NOT ED-derived.</t>
-        </is>
-      </c>
-      <c r="D406" s="41" t="inlineStr">
-        <is>
-          <t>Prediction</t>
-        </is>
-      </c>
-      <c r="E406" s="41" t="inlineStr">
-        <is>
-          <t>measured absolute nu masses with Koide combination != ~0.77 refute; untestable until absolute nu masses known</t>
-        </is>
-      </c>
-      <c r="F406" s="41" t="inlineStr">
-        <is>
-          <t>toy-map extrapolation; not derived (masses inherited)</t>
-        </is>
-      </c>
-      <c r="G406" s="41" t="inlineStr">
-        <is>
-          <t>absolute nu masses unknown; untestable now</t>
-        </is>
-      </c>
-      <c r="H406" t="inlineStr">
-        <is>
-          <t>toy-model / re-description tier (Paper_Koide_GenerationCoherenceMap)</t>
-        </is>
-      </c>
-      <c r="I406" t="inlineStr"/>
-      <c r="J406" t="inlineStr"/>
-    </row>
-    <row r="407" ht="15.75" customHeight="1" s="39">
-      <c r="A407" s="41" t="inlineStr">
-        <is>
-          <t>substrate-evaluation</t>
-        </is>
-      </c>
-      <c r="B407" s="41" t="inlineStr">
-        <is>
-          <t>Koide</t>
-        </is>
-      </c>
-      <c r="C407" s="41" t="inlineStr">
-        <is>
-          <t>Koide 2/3 re-described in ED amplitude/coherence language (mass = bandwidth b, sqrt m = amplitude): Q reads as a coherence ratio among 3 generation-amplitudes; Q = 1/3 + w^2/6; Brannen Z3 / sqrt2 form; leptons w=sqrt2, delta~2/9. RE-DESCRIPTION + consilience (masses organize like amplitudes), NOT a derivation.</t>
-        </is>
-      </c>
-      <c r="D407" s="41" t="inlineStr">
-        <is>
-          <t>Inherited / Consilience</t>
-        </is>
-      </c>
-      <c r="E407" s="41" t="inlineStr">
-        <is>
-          <t>n/a (re-description; no ED derivation to falsify)</t>
-        </is>
-      </c>
-      <c r="F407" s="41" t="inlineStr">
-        <is>
-          <t>none - re-description; mass sector inherited/open</t>
-        </is>
-      </c>
-      <c r="G407" s="41" t="inlineStr">
-        <is>
-          <t>generation count, masses, 2/3, w=sqrt2, delta~2/9 all inherited/open</t>
-        </is>
-      </c>
-      <c r="H407" t="inlineStr">
-        <is>
-          <t>referee-vetted; obeys B4 retrofit discipline; Paper_Koide_GenerationCoherenceMap</t>
-        </is>
-      </c>
-      <c r="I407" t="inlineStr"/>
-      <c r="J407" t="inlineStr"/>
-    </row>
+    <row r="406" ht="15.75" customHeight="1" s="39"/>
+    <row r="407" ht="15.75" customHeight="1" s="39"/>
     <row r="408" ht="15.75" customHeight="1" s="39"/>
     <row r="409" ht="15.75" customHeight="1" s="39"/>
     <row r="410" ht="15.75" customHeight="1" s="39"/>
@@ -18792,7 +18679,7 @@
     <row r="999" ht="15.75" customHeight="1" s="39"/>
     <row r="1000" ht="15.75" customHeight="1" s="39"/>
   </sheetData>
-  <autoFilter ref="A1:J407">
+  <autoFilter ref="A1:J405">
     <sortState ref="A1:J402">
       <sortCondition ref="D1:D402"/>
       <sortCondition ref="J1:J402"/>
@@ -24720,13 +24607,12 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A2:B8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="43.43" customWidth="1" style="39" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="A2" s="33" t="inlineStr">
         <is>
@@ -24754,7 +24640,7 @@
         </is>
       </c>
       <c r="B4" s="33" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">

</xml_diff>